<commit_message>
chore: sync local ledger storage
</commit_message>
<xml_diff>
--- a/data/ledger.xlsx
+++ b/data/ledger.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="76">
   <si>
     <t>ID</t>
   </si>
@@ -37,6 +37,9 @@
     <t>PersonName</t>
   </si>
   <si>
+    <t>ContactNumber</t>
+  </si>
+  <si>
     <t>PaymentMethod</t>
   </si>
   <si>
@@ -49,6 +52,36 @@
     <t>CreatedAt</t>
   </si>
   <si>
+    <t>tx_mvt7llq2_2jf3sgw</t>
+  </si>
+  <si>
+    <t>2026-10-29</t>
+  </si>
+  <si>
+    <t>expense</t>
+  </si>
+  <si>
+    <t>cat_6</t>
+  </si>
+  <si>
+    <t>Uncategorized</t>
+  </si>
+  <si>
+    <t>Lohith</t>
+  </si>
+  <si>
+    <t>6301865010</t>
+  </si>
+  <si>
+    <t>upi</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>2026-10-29T07:15:46.875Z</t>
+  </si>
+  <si>
     <t>Name</t>
   </si>
   <si>
@@ -97,9 +130,6 @@
     <t>Food</t>
   </si>
   <si>
-    <t>expense</t>
-  </si>
-  <si>
     <t>cat_mvsbgpoc_afa7m</t>
   </si>
   <si>
@@ -163,9 +193,6 @@
     <t>logo_url</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>opening_balance</t>
   </si>
   <si>
@@ -206,6 +233,15 @@
   </si>
   <si>
     <t>Initialized new Excel ledger workbook</t>
+  </si>
+  <si>
+    <t>INSERT</t>
+  </si>
+  <si>
+    <t>transactions</t>
+  </si>
+  <si>
+    <t>Recorded expense of ₹100 for Uncategorized</t>
   </si>
 </sst>
 </file>
@@ -586,7 +622,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:L2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -602,7 +638,7 @@
     <col min="11" max="11" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -636,10 +672,51 @@
       <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2">
+        <v>100</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L2" t="s">
+        <v>21</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -659,214 +736,214 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>11</v>
+        <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>12</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D2" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="C3" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D4" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C5" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="C6" t="s">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="C7" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>28</v>
+        <v>38</v>
       </c>
       <c r="B8" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="C9" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>32</v>
+        <v>42</v>
       </c>
       <c r="B10" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="C10" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D10" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>44</v>
       </c>
       <c r="B11" t="s">
-        <v>35</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D11" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>36</v>
+        <v>46</v>
       </c>
       <c r="B12" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="C12" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D12" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>38</v>
+        <v>48</v>
       </c>
       <c r="B13" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="C13" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D13" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B14" t="s">
-        <v>41</v>
+        <v>51</v>
       </c>
       <c r="C14" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D14" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>42</v>
+        <v>52</v>
       </c>
       <c r="B15" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
       <c r="C15" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D15" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -881,61 +958,61 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>44</v>
+        <v>54</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="B2" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>48</v>
+        <v>58</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="B4" t="s">
-        <v>51</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>61</v>
       </c>
       <c r="B5" t="s">
-        <v>53</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>63</v>
       </c>
       <c r="B6" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -950,16 +1027,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -967,20 +1044,37 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="D2" t="s">
-        <v>62</v>
+        <v>71</v>
       </c>
       <c r="E2" t="s">
-        <v>63</v>
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: modern transactions UI, color-coded status shades, quick filter tabs, and Google Sheets sync
</commit_message>
<xml_diff>
--- a/data/ledger.xlsx
+++ b/data/ledger.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="93">
   <si>
     <t>ID</t>
   </si>
@@ -82,6 +82,45 @@
     <t>2026-10-29T07:15:46.875Z</t>
   </si>
   <si>
+    <t>tx_mvwgozpw_17coklh</t>
+  </si>
+  <si>
+    <t>2026-10-31</t>
+  </si>
+  <si>
+    <t>cat_7</t>
+  </si>
+  <si>
+    <t>lucky</t>
+  </si>
+  <si>
+    <t>2026-10-31T13:53:40.052Z</t>
+  </si>
+  <si>
+    <t>tx_mvwh5juj_d2h86xu</t>
+  </si>
+  <si>
+    <t>cat_11</t>
+  </si>
+  <si>
+    <t>ravi</t>
+  </si>
+  <si>
+    <t>9848058689</t>
+  </si>
+  <si>
+    <t>2026-10-31T14:06:32.635Z</t>
+  </si>
+  <si>
+    <t>tx_mvwi3bce_k892fi8</t>
+  </si>
+  <si>
+    <t>cat_14</t>
+  </si>
+  <si>
+    <t>2026-10-31T14:32:47.919Z</t>
+  </si>
+  <si>
     <t>Name</t>
   </si>
   <si>
@@ -242,6 +281,18 @@
   </si>
   <si>
     <t>Recorded expense of ₹100 for Uncategorized</t>
+  </si>
+  <si>
+    <t>2026-10-31T13:53:40.054Z</t>
+  </si>
+  <si>
+    <t>Recorded expense of ₹120 (Paid: ₹20, Pending: ₹100) for Uncategorized</t>
+  </si>
+  <si>
+    <t>Recorded expense of ₹1000 (Paid: ₹1000, Pending: ₹0) for Uncategorized</t>
+  </si>
+  <si>
+    <t>Recorded expense of ₹500 (Paid: ₹350, Pending: ₹150) for Uncategorized</t>
   </si>
 </sst>
 </file>
@@ -622,7 +673,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -712,6 +763,120 @@
       </c>
       <c r="L2" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>23</v>
+      </c>
+      <c r="C3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3">
+        <v>120</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" t="s">
+        <v>25</v>
+      </c>
+      <c r="H3" t="s">
+        <v>18</v>
+      </c>
+      <c r="I3" t="s">
+        <v>19</v>
+      </c>
+      <c r="J3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4">
+        <v>1000</v>
+      </c>
+      <c r="E4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" t="s">
+        <v>19</v>
+      </c>
+      <c r="J4" t="s">
+        <v>20</v>
+      </c>
+      <c r="K4" t="s">
+        <v>20</v>
+      </c>
+      <c r="L4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5">
+        <v>500</v>
+      </c>
+      <c r="E5" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" t="s">
+        <v>25</v>
+      </c>
+      <c r="H5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I5" t="s">
+        <v>19</v>
+      </c>
+      <c r="J5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" t="s">
+        <v>20</v>
+      </c>
+      <c r="L5" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>
@@ -736,209 +901,209 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>23</v>
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>37</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>38</v>
       </c>
       <c r="C2" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="C3" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="C4" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="D4" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="C5" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="C7" t="s">
         <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
         <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="B9" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
         <v>14</v>
       </c>
       <c r="D9" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="B10" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="C10" t="s">
         <v>14</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="C11" t="s">
         <v>14</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>46</v>
+        <v>59</v>
       </c>
       <c r="B12" t="s">
-        <v>47</v>
+        <v>60</v>
       </c>
       <c r="C12" t="s">
         <v>14</v>
       </c>
       <c r="D12" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>48</v>
+        <v>61</v>
       </c>
       <c r="B13" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
       <c r="C13" t="s">
         <v>14</v>
       </c>
       <c r="D13" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="B14" t="s">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="C14" t="s">
         <v>14</v>
       </c>
       <c r="D14" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>52</v>
+        <v>65</v>
       </c>
       <c r="B15" t="s">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="C15" t="s">
         <v>14</v>
       </c>
       <c r="D15" t="s">
-        <v>27</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -958,23 +1123,23 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>56</v>
+        <v>69</v>
       </c>
       <c r="B2" t="s">
-        <v>57</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="B3" t="s">
         <v>20</v>
@@ -982,26 +1147,26 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>59</v>
+        <v>72</v>
       </c>
       <c r="B4" t="s">
-        <v>60</v>
+        <v>73</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="B5" t="s">
-        <v>62</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>63</v>
+        <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>64</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1012,7 +1177,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1027,16 +1192,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>66</v>
+        <v>79</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1044,16 +1209,16 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="E2" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -1064,13 +1229,64 @@
         <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="D3" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="E3" t="s">
-        <v>75</v>
+        <v>88</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D4" t="s">
+        <v>87</v>
+      </c>
+      <c r="E4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>86</v>
+      </c>
+      <c r="D5" t="s">
+        <v>87</v>
+      </c>
+      <c r="E5" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" t="s">
+        <v>87</v>
+      </c>
+      <c r="E6" t="s">
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>